<commit_message>
Complete Jada Exercise 4.A
</commit_message>
<xml_diff>
--- a/Carter_Ex3A_tables.xlsx
+++ b/Carter_Ex3A_tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jadacarter\Documents\DATA_Labs\W2_Workshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{53C3BD79-C5CE-4A12-8A23-B00B55D608A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{539F3DB2-409A-4AF5-9686-75B20C566FE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-504" yWindow="756" windowWidth="13008" windowHeight="9960" activeTab="1" xr2:uid="{BC7929A4-FA98-41BA-8ADD-C8893B418D16}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{BC7929A4-FA98-41BA-8ADD-C8893B418D16}"/>
   </bookViews>
   <sheets>
     <sheet name="Customers" sheetId="1" r:id="rId1"/>
@@ -45,76 +45,480 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
-  <si>
-    <t>Customer_ID</t>
-  </si>
-  <si>
-    <t>First_Name</t>
-  </si>
-  <si>
-    <t>Last_Name</t>
-  </si>
-  <si>
-    <t>Phone</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>Dog_ID</t>
-  </si>
-  <si>
-    <t>DogName</t>
-  </si>
-  <si>
-    <t>Breed</t>
-  </si>
-  <si>
-    <t>Age</t>
-  </si>
-  <si>
-    <t>Weight</t>
-  </si>
-  <si>
-    <t>Walker_ID</t>
-  </si>
-  <si>
-    <t>Hire_Date</t>
-  </si>
-  <si>
-    <t>Home_Address</t>
-  </si>
-  <si>
-    <t>Walk_Id</t>
-  </si>
-  <si>
-    <t>Walker_id</t>
-  </si>
-  <si>
-    <t>Walk_Date</t>
-  </si>
-  <si>
-    <t>Duration</t>
-  </si>
-  <si>
-    <t>Start_Time</t>
-  </si>
-  <si>
-    <t>Status</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="150">
+  <si>
+    <t>walk_date</t>
+  </si>
+  <si>
+    <t>start_time</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>James</t>
+  </si>
+  <si>
+    <t>Miller</t>
+  </si>
+  <si>
+    <t>555-0101</t>
+  </si>
+  <si>
+    <t>james.miller@example.com</t>
+  </si>
+  <si>
+    <t>123 Maple Street</t>
+  </si>
+  <si>
+    <t>Sarah</t>
+  </si>
+  <si>
+    <t>Johnson</t>
+  </si>
+  <si>
+    <t>555-0102</t>
+  </si>
+  <si>
+    <t>sarah.johnson@example.com</t>
+  </si>
+  <si>
+    <t>Bella</t>
+  </si>
+  <si>
+    <t>Golden Retriever</t>
+  </si>
+  <si>
+    <t>Scheduled</t>
+  </si>
+  <si>
+    <t>customer_id</t>
+  </si>
+  <si>
+    <t>first_name</t>
+  </si>
+  <si>
+    <t>last_name</t>
+  </si>
+  <si>
+    <t>phone</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>home_address</t>
+  </si>
+  <si>
+    <t>duration_minutes</t>
+  </si>
+  <si>
+    <t>walker_id</t>
+  </si>
+  <si>
+    <t>dog_id</t>
+  </si>
+  <si>
+    <t>walk_id</t>
+  </si>
+  <si>
+    <t>age</t>
+  </si>
+  <si>
+    <t>breed</t>
+  </si>
+  <si>
+    <t>dog_name</t>
+  </si>
+  <si>
+    <t>dog_in</t>
+  </si>
+  <si>
+    <t>Olivia</t>
+  </si>
+  <si>
+    <t>Reed</t>
+  </si>
+  <si>
+    <t>olivia.reed@example.com</t>
+  </si>
+  <si>
+    <t>45 Oak Avenue</t>
+  </si>
+  <si>
+    <t>Noah</t>
+  </si>
+  <si>
+    <t>Brooks</t>
+  </si>
+  <si>
+    <t>555-0103</t>
+  </si>
+  <si>
+    <t>noah.brooks@example.com</t>
+  </si>
+  <si>
+    <t>78 Pine Road</t>
+  </si>
+  <si>
+    <t>Emma</t>
+  </si>
+  <si>
+    <t>Davis</t>
+  </si>
+  <si>
+    <t>555-0104</t>
+  </si>
+  <si>
+    <t>emma.davis@example.com</t>
+  </si>
+  <si>
+    <t>12 Cedar Lane</t>
+  </si>
+  <si>
+    <t>Liam</t>
+  </si>
+  <si>
+    <t>Carter</t>
+  </si>
+  <si>
+    <t>555-0105</t>
+  </si>
+  <si>
+    <t>liam.carter@example.com</t>
+  </si>
+  <si>
+    <t>90 Birch Drive</t>
+  </si>
+  <si>
+    <t>Ava</t>
+  </si>
+  <si>
+    <t>Thompson</t>
+  </si>
+  <si>
+    <t>555-0106</t>
+  </si>
+  <si>
+    <t>ava.thompson@example.com</t>
+  </si>
+  <si>
+    <t>34 Willow Street</t>
+  </si>
+  <si>
+    <t>Ethan</t>
+  </si>
+  <si>
+    <t>Parker</t>
+  </si>
+  <si>
+    <t>555-0107</t>
+  </si>
+  <si>
+    <t>ethan.parker@example.com</t>
+  </si>
+  <si>
+    <t>67 Elm Avenue</t>
+  </si>
+  <si>
+    <t>Mia</t>
+  </si>
+  <si>
+    <t>Flores</t>
+  </si>
+  <si>
+    <t>555-0108</t>
+  </si>
+  <si>
+    <t>mia.flores@example.com</t>
+  </si>
+  <si>
+    <t>81 Cherry Lane</t>
+  </si>
+  <si>
+    <t>Lucas</t>
+  </si>
+  <si>
+    <t>Bennett</t>
+  </si>
+  <si>
+    <t>555-0109</t>
+  </si>
+  <si>
+    <t>lucas.bennett@example.com</t>
+  </si>
+  <si>
+    <t>56 Walnut Road</t>
+  </si>
+  <si>
+    <t>Sophia</t>
+  </si>
+  <si>
+    <t>Green</t>
+  </si>
+  <si>
+    <t>555-0110</t>
+  </si>
+  <si>
+    <t>sophia.green@example.com</t>
+  </si>
+  <si>
+    <t>23 Aspen Street</t>
+  </si>
+  <si>
+    <t>Mason</t>
+  </si>
+  <si>
+    <t>Collins</t>
+  </si>
+  <si>
+    <t>555-0111</t>
+  </si>
+  <si>
+    <t>mason.collins@example.com</t>
+  </si>
+  <si>
+    <t>102 Spruce Drive</t>
+  </si>
+  <si>
+    <t>Daniel</t>
+  </si>
+  <si>
+    <t>Ruiz</t>
+  </si>
+  <si>
+    <t>555-0202</t>
+  </si>
+  <si>
+    <t>daniel.ruiz@example.com</t>
+  </si>
+  <si>
+    <t>Emily</t>
+  </si>
+  <si>
+    <t>Foster</t>
+  </si>
+  <si>
+    <t>555-0203</t>
+  </si>
+  <si>
+    <t>emily.foster@example.com</t>
+  </si>
+  <si>
+    <t>Marcus</t>
+  </si>
+  <si>
+    <t>Lee</t>
+  </si>
+  <si>
+    <t>555-0204</t>
+  </si>
+  <si>
+    <t>marcus.lee@example.com</t>
+  </si>
+  <si>
+    <t>Rachel</t>
+  </si>
+  <si>
+    <t>Kim</t>
+  </si>
+  <si>
+    <t>555-0205</t>
+  </si>
+  <si>
+    <t>rachel.kim@example.com</t>
+  </si>
+  <si>
+    <t>Tyler</t>
+  </si>
+  <si>
+    <t>Adams</t>
+  </si>
+  <si>
+    <t>555-0206</t>
+  </si>
+  <si>
+    <t>tyler.adams@example.com</t>
+  </si>
+  <si>
+    <t>Hannah</t>
+  </si>
+  <si>
+    <t>555-0207</t>
+  </si>
+  <si>
+    <t>hannah.brooks@example.com</t>
+  </si>
+  <si>
+    <t>David</t>
+  </si>
+  <si>
+    <t>Chen</t>
+  </si>
+  <si>
+    <t>555-0208</t>
+  </si>
+  <si>
+    <t>david.chen@example.com</t>
+  </si>
+  <si>
+    <t>Nicole</t>
+  </si>
+  <si>
+    <t>Wright</t>
+  </si>
+  <si>
+    <t>555-0209</t>
+  </si>
+  <si>
+    <t>nicole.wright@example.com</t>
+  </si>
+  <si>
+    <t>Jordan</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>555-0210</t>
+  </si>
+  <si>
+    <t>jordan.price@example.com</t>
+  </si>
+  <si>
+    <t>Chloe</t>
+  </si>
+  <si>
+    <t>Rivera</t>
+  </si>
+  <si>
+    <t>555-0211</t>
+  </si>
+  <si>
+    <t>chloe.rivera@example.com</t>
+  </si>
+  <si>
+    <t>specail_instructions</t>
+  </si>
+  <si>
+    <t>Max</t>
+  </si>
+  <si>
+    <t>German Shepherd</t>
+  </si>
+  <si>
+    <t>Prefers quiet walking routes</t>
+  </si>
+  <si>
+    <t>Luna</t>
+  </si>
+  <si>
+    <t>Labrador Retriever</t>
+  </si>
+  <si>
+    <t>Very energetic</t>
+  </si>
+  <si>
+    <t>Charlie</t>
+  </si>
+  <si>
+    <t>Beagle</t>
+  </si>
+  <si>
+    <t>Keep away from busy roads</t>
+  </si>
+  <si>
+    <t>Daisy</t>
+  </si>
+  <si>
+    <t>Poodle</t>
+  </si>
+  <si>
+    <t>Walk at a slower pace</t>
+  </si>
+  <si>
+    <t>Rocky</t>
+  </si>
+  <si>
+    <t>Bulldog</t>
+  </si>
+  <si>
+    <t>Avoid long walks in hot weather</t>
+  </si>
+  <si>
+    <t>Coco</t>
+  </si>
+  <si>
+    <t>Chihuahua</t>
+  </si>
+  <si>
+    <t>Gets nervous around large dogs</t>
+  </si>
+  <si>
+    <t>Milo</t>
+  </si>
+  <si>
+    <t>Border Collie</t>
+  </si>
+  <si>
+    <t>Needs plenty of exercise</t>
+  </si>
+  <si>
+    <t>Bailey</t>
+  </si>
+  <si>
+    <t>Still learning leash manners</t>
+  </si>
+  <si>
+    <t>Ruby</t>
+  </si>
+  <si>
+    <t>Boxer</t>
+  </si>
+  <si>
+    <t>Loves outdoor activities</t>
+  </si>
+  <si>
+    <t>Teddy</t>
+  </si>
+  <si>
+    <t>Shih Tzu</t>
+  </si>
+  <si>
+    <t>Short walks preferred</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>Cancelled</t>
+  </si>
+  <si>
+    <t>friendly, needs water breaks</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Inherit"/>
     </font>
   </fonts>
   <fills count="4">
@@ -149,10 +553,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -487,134 +897,1029 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C7E9E0B-8D43-4A2F-92AE-29782D34E4DA}">
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="11.109375" customWidth="1"/>
     <col min="2" max="2" width="9.77734375" customWidth="1"/>
-    <col min="3" max="3" width="9.6640625" customWidth="1"/>
-    <col min="6" max="6" width="13.33203125" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" customWidth="1"/>
+    <col min="4" max="4" width="12.21875" customWidth="1"/>
+    <col min="5" max="5" width="25" customWidth="1"/>
+    <col min="6" max="6" width="14.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="B1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="B3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="B4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
-        <v>12</v>
+      <c r="B5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E5" t="s">
+        <v>41</v>
+      </c>
+      <c r="F5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E6" t="s">
+        <v>46</v>
+      </c>
+      <c r="F6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E7" t="s">
+        <v>51</v>
+      </c>
+      <c r="F7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" t="s">
+        <v>55</v>
+      </c>
+      <c r="E8" t="s">
+        <v>56</v>
+      </c>
+      <c r="F8" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9" t="s">
+        <v>60</v>
+      </c>
+      <c r="E9" t="s">
+        <v>61</v>
+      </c>
+      <c r="F9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" t="s">
+        <v>64</v>
+      </c>
+      <c r="D10" t="s">
+        <v>65</v>
+      </c>
+      <c r="E10" t="s">
+        <v>66</v>
+      </c>
+      <c r="F10" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>68</v>
+      </c>
+      <c r="C11" t="s">
+        <v>69</v>
+      </c>
+      <c r="D11" t="s">
+        <v>70</v>
+      </c>
+      <c r="E11" t="s">
+        <v>71</v>
+      </c>
+      <c r="F11" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C12" t="s">
+        <v>74</v>
+      </c>
+      <c r="D12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E12" t="s">
+        <v>76</v>
+      </c>
+      <c r="F12" t="s">
+        <v>77</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBBBA6E9-3BE2-4DD6-97FF-F5E4564D9BC8}">
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="11.88671875" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" customWidth="1"/>
+    <col min="6" max="6" width="26.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2">
+        <v>3</v>
+      </c>
+      <c r="F2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>118</v>
+      </c>
+      <c r="D3" t="s">
+        <v>119</v>
+      </c>
+      <c r="E3">
         <v>5</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="F3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>121</v>
+      </c>
+      <c r="D4" t="s">
+        <v>122</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D5" t="s">
+        <v>125</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>127</v>
+      </c>
+      <c r="D6" t="s">
+        <v>128</v>
+      </c>
+      <c r="E6">
         <v>6</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F6" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>6</v>
+      </c>
+      <c r="C7" t="s">
+        <v>130</v>
+      </c>
+      <c r="D7" t="s">
+        <v>131</v>
+      </c>
+      <c r="E7">
+        <v>3</v>
+      </c>
+      <c r="F7" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8">
         <v>7</v>
       </c>
-      <c r="E1" t="s">
+      <c r="B8">
+        <v>7</v>
+      </c>
+      <c r="C8" t="s">
+        <v>133</v>
+      </c>
+      <c r="D8" t="s">
+        <v>134</v>
+      </c>
+      <c r="E8">
+        <v>7</v>
+      </c>
+      <c r="F8" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9">
         <v>8</v>
       </c>
-      <c r="F1" t="s">
+      <c r="B9">
+        <v>8</v>
+      </c>
+      <c r="C9" t="s">
+        <v>136</v>
+      </c>
+      <c r="D9" t="s">
+        <v>137</v>
+      </c>
+      <c r="E9">
+        <v>2</v>
+      </c>
+      <c r="F9" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10">
         <v>9</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>139</v>
+      </c>
+      <c r="D10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>9</v>
+      </c>
+      <c r="C11" t="s">
+        <v>141</v>
+      </c>
+      <c r="D11" t="s">
+        <v>142</v>
+      </c>
+      <c r="E11">
+        <v>4</v>
+      </c>
+      <c r="F11" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>10</v>
+      </c>
+      <c r="C12" t="s">
+        <v>144</v>
+      </c>
+      <c r="D12" t="s">
+        <v>145</v>
+      </c>
+      <c r="E12">
+        <v>5</v>
+      </c>
+      <c r="F12" t="s">
+        <v>146</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E1AD1E8-5F9D-46D4-B632-2F16B7B01229}">
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="2" max="2" width="10.6640625" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="5" max="5" width="25.109375" customWidth="1"/>
+    <col min="6" max="6" width="26" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
         <v>10</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="B3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D3" t="s">
+        <v>80</v>
+      </c>
+      <c r="E3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="B4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4" t="s">
+        <v>83</v>
+      </c>
+      <c r="D4" t="s">
+        <v>84</v>
+      </c>
+      <c r="E4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>86</v>
+      </c>
+      <c r="C5" t="s">
+        <v>87</v>
+      </c>
+      <c r="D5" t="s">
+        <v>88</v>
+      </c>
+      <c r="E5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D6" t="s">
+        <v>92</v>
+      </c>
+      <c r="E6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="4">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>94</v>
+      </c>
+      <c r="C7" t="s">
+        <v>95</v>
+      </c>
+      <c r="D7" t="s">
+        <v>96</v>
+      </c>
+      <c r="E7" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" t="s">
+        <v>99</v>
+      </c>
+      <c r="E8" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>101</v>
+      </c>
+      <c r="C9" t="s">
+        <v>102</v>
+      </c>
+      <c r="D9" t="s">
+        <v>103</v>
+      </c>
+      <c r="E9" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>105</v>
+      </c>
+      <c r="C10" t="s">
+        <v>106</v>
+      </c>
+      <c r="D10" t="s">
+        <v>107</v>
+      </c>
+      <c r="E10" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>109</v>
+      </c>
+      <c r="C11" t="s">
+        <v>110</v>
+      </c>
+      <c r="D11" t="s">
+        <v>111</v>
+      </c>
+      <c r="E11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12">
         <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>113</v>
+      </c>
+      <c r="C12" t="s">
+        <v>114</v>
+      </c>
+      <c r="D12" t="s">
+        <v>115</v>
+      </c>
+      <c r="E12" t="s">
+        <v>116</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD08CCEA-D957-4A09-852F-47B3234030CB}">
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
-    <col min="4" max="4" width="9.88671875" customWidth="1"/>
-    <col min="5" max="5" width="9.5546875" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.5546875" customWidth="1"/>
+    <col min="6" max="6" width="16.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" s="5">
+        <v>46318</v>
+      </c>
+      <c r="E2" s="6">
+        <v>46318.375</v>
+      </c>
+      <c r="F2">
+        <v>30</v>
+      </c>
+      <c r="G2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3" s="5">
+        <v>46314</v>
+      </c>
+      <c r="E3" s="6">
+        <v>46314.354166666664</v>
+      </c>
+      <c r="F3">
+        <v>45</v>
+      </c>
+      <c r="G3" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4" s="5">
+        <v>46315</v>
+      </c>
+      <c r="E4" s="6">
+        <v>46315.5</v>
+      </c>
+      <c r="F4">
+        <v>30</v>
+      </c>
+      <c r="G4" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" s="5">
+        <v>46316</v>
+      </c>
+      <c r="E5" s="6">
+        <v>46316.427083333336</v>
+      </c>
+      <c r="F5">
+        <v>60</v>
+      </c>
+      <c r="G5" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6">
         <v>5</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6" s="5">
+        <v>46319</v>
+      </c>
+      <c r="E6" s="6">
+        <v>46319.458333333336</v>
+      </c>
+      <c r="F6">
+        <v>30</v>
+      </c>
+      <c r="G6" t="s">
         <v>14</v>
       </c>
-      <c r="D1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F1" t="s">
-        <v>16</v>
-      </c>
-      <c r="G1" t="s">
-        <v>18</v>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>6</v>
+      </c>
+      <c r="C7">
+        <v>4</v>
+      </c>
+      <c r="D7" s="5">
+        <v>46320</v>
+      </c>
+      <c r="E7" s="6">
+        <v>46320.583333333336</v>
+      </c>
+      <c r="F7">
+        <v>45</v>
+      </c>
+      <c r="G7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>7</v>
+      </c>
+      <c r="C8">
+        <v>5</v>
+      </c>
+      <c r="D8" s="5">
+        <v>46313</v>
+      </c>
+      <c r="E8" s="6">
+        <v>46313.395833333336</v>
+      </c>
+      <c r="F8">
+        <v>30</v>
+      </c>
+      <c r="G8" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>8</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9" s="5">
+        <v>46321</v>
+      </c>
+      <c r="E9" s="6">
+        <v>46321.666666666664</v>
+      </c>
+      <c r="F9">
+        <v>45</v>
+      </c>
+      <c r="G9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>9</v>
+      </c>
+      <c r="C10">
+        <v>3</v>
+      </c>
+      <c r="D10" s="5">
+        <v>46312</v>
+      </c>
+      <c r="E10" s="6">
+        <v>46312.541666666664</v>
+      </c>
+      <c r="F10">
+        <v>30</v>
+      </c>
+      <c r="G10" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>10</v>
+      </c>
+      <c r="C11">
+        <v>4</v>
+      </c>
+      <c r="D11" s="5">
+        <v>46322</v>
+      </c>
+      <c r="E11" s="6">
+        <v>46322.333333333336</v>
+      </c>
+      <c r="F11">
+        <v>60</v>
+      </c>
+      <c r="G11" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>11</v>
+      </c>
+      <c r="C12">
+        <v>2</v>
+      </c>
+      <c r="D12" s="5">
+        <v>46323</v>
+      </c>
+      <c r="E12" s="6">
+        <v>46323.645833333336</v>
+      </c>
+      <c r="F12">
+        <v>30</v>
+      </c>
+      <c r="G12" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>